<commit_message>
fix: distribution exportation issues
</commit_message>
<xml_diff>
--- a/SupervisorMobility.API/DataAccess/Templates/Distribution Extra Template.xlsx
+++ b/SupervisorMobility.API/DataAccess/Templates/Distribution Extra Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ituriel\OneDrive\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C94CE4E-6DA1-4B24-B4E0-A306E946BA83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6BC41ED-A41F-44CC-B095-6FDECBDE29FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="52740" yWindow="4365" windowWidth="23235" windowHeight="10950" xr2:uid="{4D8E7E08-F2C9-45F6-938C-67D482DEBE58}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="18672" windowHeight="10320" xr2:uid="{4D8E7E08-F2C9-45F6-938C-67D482DEBE58}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -604,11 +604,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -659,6 +657,36 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -734,46 +762,34 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1128,219 +1144,214 @@
   <sheetData>
     <row r="1" spans="2:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="32"/>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
-      <c r="N2" s="32"/>
-      <c r="O2" s="32"/>
-      <c r="P2" s="32"/>
-      <c r="Q2" s="32"/>
-      <c r="R2" s="32"/>
-      <c r="S2" s="32"/>
-      <c r="T2" s="32"/>
-      <c r="U2" s="32"/>
-      <c r="V2" s="32"/>
-      <c r="W2" s="32"/>
-      <c r="X2" s="32"/>
-      <c r="Y2" s="32"/>
-      <c r="Z2" s="32"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
+      <c r="I2" s="40"/>
+      <c r="J2" s="40"/>
+      <c r="K2" s="40"/>
+      <c r="L2" s="40"/>
+      <c r="M2" s="40"/>
+      <c r="N2" s="40"/>
+      <c r="O2" s="40"/>
+      <c r="P2" s="40"/>
+      <c r="Q2" s="40"/>
+      <c r="R2" s="40"/>
+      <c r="S2" s="40"/>
+      <c r="T2" s="40"/>
+      <c r="U2" s="40"/>
+      <c r="V2" s="40"/>
+      <c r="W2" s="40"/>
+      <c r="X2" s="40"/>
+      <c r="Y2" s="40"/>
+      <c r="Z2" s="40"/>
     </row>
     <row r="3" spans="2:26" ht="6.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="2:26" ht="6.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="2:26" ht="9.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="6" spans="2:26" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="U6" s="21"/>
-      <c r="V6" s="20" t="s">
+      <c r="U6" s="19"/>
+      <c r="V6" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="W6" s="22"/>
+      <c r="W6" s="20"/>
     </row>
     <row r="7" spans="2:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="54" t="s">
+      <c r="B7" s="56" t="s">
         <v>0</v>
       </c>
-      <c r="C7" s="56" t="s">
+      <c r="C7" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="57"/>
-      <c r="E7" s="57"/>
-      <c r="F7" s="57"/>
-      <c r="G7" s="58"/>
-      <c r="H7" s="56" t="s">
+      <c r="D7" s="22"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="22"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="I7" s="57"/>
-      <c r="J7" s="57"/>
-      <c r="K7" s="58"/>
-      <c r="L7" s="62" t="s">
+      <c r="I7" s="22"/>
+      <c r="J7" s="22"/>
+      <c r="K7" s="23"/>
+      <c r="L7" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="M7" s="63"/>
-      <c r="N7" s="63"/>
-      <c r="O7" s="63"/>
-      <c r="P7" s="63"/>
-      <c r="Q7" s="56" t="s">
+      <c r="M7" s="28"/>
+      <c r="N7" s="28"/>
+      <c r="O7" s="28"/>
+      <c r="P7" s="28"/>
+      <c r="Q7" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="R7" s="57"/>
-      <c r="S7" s="57"/>
-      <c r="T7" s="57"/>
-      <c r="U7" s="57"/>
-      <c r="V7" s="57"/>
-      <c r="W7" s="64"/>
+      <c r="R7" s="22"/>
+      <c r="S7" s="22"/>
+      <c r="T7" s="22"/>
+      <c r="U7" s="22"/>
+      <c r="V7" s="22"/>
+      <c r="W7" s="29"/>
     </row>
     <row r="8" spans="2:26" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="55"/>
-      <c r="C8" s="59" t="s">
+      <c r="B8" s="57"/>
+      <c r="C8" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="D8" s="60"/>
-      <c r="E8" s="60"/>
-      <c r="F8" s="60"/>
-      <c r="G8" s="61"/>
-      <c r="H8" s="59"/>
-      <c r="I8" s="60"/>
-      <c r="J8" s="60"/>
-      <c r="K8" s="61"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="25"/>
+      <c r="F8" s="25"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="24"/>
+      <c r="I8" s="25"/>
+      <c r="J8" s="25"/>
+      <c r="K8" s="26"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
       <c r="O8" s="2"/>
       <c r="P8" s="2"/>
-      <c r="Q8" s="59"/>
-      <c r="R8" s="60"/>
-      <c r="S8" s="60"/>
-      <c r="T8" s="60"/>
-      <c r="U8" s="60"/>
-      <c r="V8" s="60"/>
-      <c r="W8" s="65"/>
+      <c r="Q8" s="24"/>
+      <c r="R8" s="25"/>
+      <c r="S8" s="25"/>
+      <c r="T8" s="25"/>
+      <c r="U8" s="25"/>
+      <c r="V8" s="25"/>
+      <c r="W8" s="30"/>
     </row>
     <row r="9" spans="2:26" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="3"/>
-      <c r="C9" s="48"/>
-      <c r="D9" s="49"/>
-      <c r="E9" s="49"/>
-      <c r="F9" s="49"/>
-      <c r="G9" s="50"/>
-      <c r="H9" s="48"/>
-      <c r="I9" s="49"/>
-      <c r="J9" s="49"/>
-      <c r="K9" s="50"/>
-      <c r="L9" s="4"/>
-      <c r="M9" s="4"/>
-      <c r="N9" s="4"/>
-      <c r="O9" s="4"/>
-      <c r="P9" s="4"/>
-      <c r="W9" s="19"/>
+      <c r="B9" s="64"/>
+      <c r="C9" s="58"/>
+      <c r="D9" s="59"/>
+      <c r="E9" s="59"/>
+      <c r="F9" s="59"/>
+      <c r="G9" s="60"/>
+      <c r="H9" s="58"/>
+      <c r="I9" s="59"/>
+      <c r="J9" s="59"/>
+      <c r="K9" s="60"/>
+      <c r="L9" s="3"/>
+      <c r="M9" s="3"/>
+      <c r="N9" s="3"/>
+      <c r="O9" s="3"/>
+      <c r="P9" s="3"/>
+      <c r="W9" s="17"/>
     </row>
     <row r="10" spans="2:26" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="5"/>
-      <c r="C10" s="51"/>
-      <c r="D10" s="52"/>
-      <c r="E10" s="52"/>
-      <c r="F10" s="52"/>
-      <c r="G10" s="53"/>
-      <c r="H10" s="51"/>
-      <c r="I10" s="52"/>
-      <c r="J10" s="52"/>
-      <c r="K10" s="53"/>
-      <c r="L10" s="6"/>
-      <c r="M10" s="7"/>
-      <c r="N10" s="7"/>
-      <c r="O10" s="16"/>
-      <c r="P10" s="8"/>
-      <c r="Q10" s="33" t="s">
+      <c r="B10" s="65"/>
+      <c r="C10" s="61"/>
+      <c r="D10" s="62"/>
+      <c r="E10" s="62"/>
+      <c r="F10" s="62"/>
+      <c r="G10" s="63"/>
+      <c r="H10" s="61"/>
+      <c r="I10" s="62"/>
+      <c r="J10" s="62"/>
+      <c r="K10" s="63"/>
+      <c r="L10" s="4"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="5"/>
+      <c r="O10" s="14"/>
+      <c r="P10" s="6"/>
+      <c r="Q10" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="R10" s="9" t="s">
+      <c r="R10" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="S10" s="10" t="s">
+      <c r="S10" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="T10" s="9" t="s">
+      <c r="T10" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="U10" s="11" t="s">
+      <c r="U10" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="V10" s="26" t="s">
+      <c r="V10" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="W10" s="27"/>
+      <c r="W10" s="35"/>
     </row>
     <row r="11" spans="2:26" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="36" t="s">
+      <c r="B11" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="37"/>
-      <c r="D11" s="37"/>
-      <c r="E11" s="38"/>
-      <c r="F11" s="42" t="s">
+      <c r="C11" s="45"/>
+      <c r="D11" s="45"/>
+      <c r="E11" s="46"/>
+      <c r="F11" s="50" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="43"/>
-      <c r="H11" s="43"/>
-      <c r="I11" s="43"/>
-      <c r="J11" s="43"/>
-      <c r="K11" s="44"/>
-      <c r="L11" s="12"/>
-      <c r="M11" s="12"/>
-      <c r="N11" s="13"/>
-      <c r="O11" s="17"/>
-      <c r="P11" s="14"/>
-      <c r="Q11" s="34"/>
-      <c r="R11" s="45"/>
-      <c r="S11" s="47"/>
-      <c r="T11" s="45"/>
-      <c r="U11" s="45"/>
-      <c r="V11" s="28"/>
-      <c r="W11" s="29"/>
+      <c r="G11" s="51"/>
+      <c r="H11" s="51"/>
+      <c r="I11" s="51"/>
+      <c r="J11" s="51"/>
+      <c r="K11" s="52"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="11"/>
+      <c r="O11" s="15"/>
+      <c r="P11" s="12"/>
+      <c r="Q11" s="42"/>
+      <c r="R11" s="53"/>
+      <c r="S11" s="55"/>
+      <c r="T11" s="53"/>
+      <c r="U11" s="53"/>
+      <c r="V11" s="36"/>
+      <c r="W11" s="37"/>
     </row>
     <row r="12" spans="2:26" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="39"/>
-      <c r="C12" s="40"/>
-      <c r="D12" s="40"/>
-      <c r="E12" s="41"/>
-      <c r="F12" s="23" t="s">
+      <c r="B12" s="47"/>
+      <c r="C12" s="48"/>
+      <c r="D12" s="48"/>
+      <c r="E12" s="49"/>
+      <c r="F12" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="G12" s="24"/>
-      <c r="H12" s="24"/>
-      <c r="I12" s="24"/>
-      <c r="J12" s="24"/>
-      <c r="K12" s="25"/>
-      <c r="L12" s="12"/>
-      <c r="M12" s="15"/>
-      <c r="N12" s="12"/>
-      <c r="O12" s="18"/>
-      <c r="P12" s="14"/>
-      <c r="Q12" s="35"/>
-      <c r="R12" s="46"/>
-      <c r="S12" s="30"/>
-      <c r="T12" s="46"/>
-      <c r="U12" s="46"/>
-      <c r="V12" s="30"/>
-      <c r="W12" s="31"/>
+      <c r="G12" s="32"/>
+      <c r="H12" s="32"/>
+      <c r="I12" s="32"/>
+      <c r="J12" s="32"/>
+      <c r="K12" s="33"/>
+      <c r="L12" s="10"/>
+      <c r="M12" s="13"/>
+      <c r="N12" s="10"/>
+      <c r="O12" s="16"/>
+      <c r="P12" s="12"/>
+      <c r="Q12" s="43"/>
+      <c r="R12" s="54"/>
+      <c r="S12" s="38"/>
+      <c r="T12" s="54"/>
+      <c r="U12" s="54"/>
+      <c r="V12" s="38"/>
+      <c r="W12" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="H7:K8"/>
-    <mergeCell ref="L7:P7"/>
-    <mergeCell ref="Q7:W8"/>
-    <mergeCell ref="C8:G8"/>
     <mergeCell ref="F12:K12"/>
     <mergeCell ref="V10:W10"/>
     <mergeCell ref="V11:W12"/>
@@ -1357,6 +1368,11 @@
     <mergeCell ref="C10:G10"/>
     <mergeCell ref="H10:K10"/>
     <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="H7:K8"/>
+    <mergeCell ref="L7:P7"/>
+    <mergeCell ref="Q7:W8"/>
+    <mergeCell ref="C8:G8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: updates do distribution exportations
</commit_message>
<xml_diff>
--- a/SupervisorMobility.API/DataAccess/Templates/Distribution Extra Template.xlsx
+++ b/SupervisorMobility.API/DataAccess/Templates/Distribution Extra Template.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ituriel\OneDrive\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\job\Supervisor app\Server\SupervisorMobility.API\DataAccess\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45DCA089-66C2-4341-9667-9AA2B0DE4853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{585F8180-E016-4695-A8B8-376D280A0AC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41595" yWindow="4425" windowWidth="31035" windowHeight="15300" xr2:uid="{4D8E7E08-F2C9-45F6-938C-67D482DEBE58}"/>
+    <workbookView xWindow="41235" yWindow="5670" windowWidth="19890" windowHeight="12300" xr2:uid="{4D8E7E08-F2C9-45F6-938C-67D482DEBE58}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -665,31 +665,118 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -705,93 +792,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1016,22 +1016,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>149263</xdr:colOff>
+      <xdr:colOff>139212</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>224006</xdr:rowOff>
+      <xdr:rowOff>212480</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>437082</xdr:colOff>
+      <xdr:colOff>425195</xdr:colOff>
       <xdr:row>11</xdr:row>
-      <xdr:rowOff>143400</xdr:rowOff>
+      <xdr:rowOff>140788</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4DEA4705-0CFD-46FD-F3F3-5B78CFFEBC96}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8EB0D3BC-50D6-4825-9D16-71B69BD56670}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1053,8 +1053,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12021895" y="2386741"/>
-          <a:ext cx="489525" cy="272380"/>
+          <a:off x="12001500" y="2395903"/>
+          <a:ext cx="483810" cy="280000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1383,6 +1383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B8E1F78-90EA-4584-8BE4-AE941805E825}">
+  <sheetPr codeName="Sheet1"/>
   <dimension ref="B1:Z12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1401,33 +1402,33 @@
   <sheetData>
     <row r="1" spans="2:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
-      <c r="G2" s="37"/>
-      <c r="H2" s="37"/>
-      <c r="I2" s="37"/>
-      <c r="J2" s="37"/>
-      <c r="K2" s="37"/>
-      <c r="L2" s="37"/>
-      <c r="M2" s="37"/>
-      <c r="N2" s="37"/>
-      <c r="O2" s="37"/>
-      <c r="P2" s="37"/>
-      <c r="Q2" s="37"/>
-      <c r="R2" s="37"/>
-      <c r="S2" s="37"/>
-      <c r="T2" s="37"/>
-      <c r="U2" s="37"/>
-      <c r="V2" s="37"/>
-      <c r="W2" s="37"/>
-      <c r="X2" s="37"/>
-      <c r="Y2" s="37"/>
-      <c r="Z2" s="37"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
+      <c r="K2" s="23"/>
+      <c r="L2" s="23"/>
+      <c r="M2" s="23"/>
+      <c r="N2" s="23"/>
+      <c r="O2" s="23"/>
+      <c r="P2" s="23"/>
+      <c r="Q2" s="23"/>
+      <c r="R2" s="23"/>
+      <c r="S2" s="23"/>
+      <c r="T2" s="23"/>
+      <c r="U2" s="23"/>
+      <c r="V2" s="23"/>
+      <c r="W2" s="23"/>
+      <c r="X2" s="23"/>
+      <c r="Y2" s="23"/>
+      <c r="Z2" s="23"/>
     </row>
     <row r="3" spans="2:26" ht="6.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="2:26" ht="6.75" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -1440,76 +1441,76 @@
       <c r="W6" s="19"/>
     </row>
     <row r="7" spans="2:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="60" t="s">
+      <c r="B7" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="51" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="26"/>
-      <c r="E7" s="26"/>
-      <c r="F7" s="26"/>
-      <c r="G7" s="65"/>
-      <c r="H7" s="25" t="s">
+      <c r="D7" s="52"/>
+      <c r="E7" s="52"/>
+      <c r="F7" s="52"/>
+      <c r="G7" s="53"/>
+      <c r="H7" s="51" t="s">
         <v>4</v>
       </c>
-      <c r="I7" s="26"/>
-      <c r="J7" s="26"/>
-      <c r="K7" s="65"/>
-      <c r="L7" s="23" t="s">
+      <c r="I7" s="52"/>
+      <c r="J7" s="52"/>
+      <c r="K7" s="53"/>
+      <c r="L7" s="57" t="s">
         <v>5</v>
       </c>
-      <c r="M7" s="24"/>
-      <c r="N7" s="24"/>
-      <c r="O7" s="24"/>
-      <c r="P7" s="24"/>
-      <c r="Q7" s="25" t="s">
+      <c r="M7" s="58"/>
+      <c r="N7" s="58"/>
+      <c r="O7" s="58"/>
+      <c r="P7" s="58"/>
+      <c r="Q7" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="R7" s="26"/>
-      <c r="S7" s="26"/>
-      <c r="T7" s="26"/>
-      <c r="U7" s="26"/>
-      <c r="V7" s="26"/>
-      <c r="W7" s="27"/>
+      <c r="R7" s="52"/>
+      <c r="S7" s="52"/>
+      <c r="T7" s="52"/>
+      <c r="U7" s="52"/>
+      <c r="V7" s="52"/>
+      <c r="W7" s="59"/>
     </row>
     <row r="8" spans="2:26" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="61"/>
-      <c r="C8" s="28" t="s">
+      <c r="B8" s="47"/>
+      <c r="C8" s="54" t="s">
         <v>7</v>
       </c>
-      <c r="D8" s="29"/>
-      <c r="E8" s="29"/>
-      <c r="F8" s="29"/>
-      <c r="G8" s="31"/>
-      <c r="H8" s="28"/>
-      <c r="I8" s="29"/>
-      <c r="J8" s="29"/>
-      <c r="K8" s="31"/>
+      <c r="D8" s="55"/>
+      <c r="E8" s="55"/>
+      <c r="F8" s="55"/>
+      <c r="G8" s="56"/>
+      <c r="H8" s="54"/>
+      <c r="I8" s="55"/>
+      <c r="J8" s="55"/>
+      <c r="K8" s="56"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
       <c r="O8" s="2"/>
       <c r="P8" s="2"/>
-      <c r="Q8" s="28"/>
-      <c r="R8" s="29"/>
-      <c r="S8" s="29"/>
-      <c r="T8" s="29"/>
-      <c r="U8" s="29"/>
-      <c r="V8" s="29"/>
-      <c r="W8" s="30"/>
+      <c r="Q8" s="54"/>
+      <c r="R8" s="55"/>
+      <c r="S8" s="55"/>
+      <c r="T8" s="55"/>
+      <c r="U8" s="55"/>
+      <c r="V8" s="55"/>
+      <c r="W8" s="60"/>
     </row>
     <row r="9" spans="2:26" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" s="20"/>
-      <c r="C9" s="54"/>
-      <c r="D9" s="55"/>
-      <c r="E9" s="55"/>
-      <c r="F9" s="55"/>
-      <c r="G9" s="56"/>
-      <c r="H9" s="54"/>
-      <c r="I9" s="55"/>
-      <c r="J9" s="55"/>
-      <c r="K9" s="56"/>
+      <c r="C9" s="40"/>
+      <c r="D9" s="41"/>
+      <c r="E9" s="41"/>
+      <c r="F9" s="41"/>
+      <c r="G9" s="42"/>
+      <c r="H9" s="40"/>
+      <c r="I9" s="41"/>
+      <c r="J9" s="41"/>
+      <c r="K9" s="42"/>
       <c r="L9" s="3"/>
       <c r="M9" s="3"/>
       <c r="N9" s="3"/>
@@ -1519,21 +1520,21 @@
     </row>
     <row r="10" spans="2:26" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="21"/>
-      <c r="C10" s="57"/>
-      <c r="D10" s="58"/>
-      <c r="E10" s="58"/>
-      <c r="F10" s="58"/>
-      <c r="G10" s="59"/>
-      <c r="H10" s="57"/>
-      <c r="I10" s="58"/>
-      <c r="J10" s="58"/>
-      <c r="K10" s="59"/>
+      <c r="C10" s="43"/>
+      <c r="D10" s="44"/>
+      <c r="E10" s="44"/>
+      <c r="F10" s="44"/>
+      <c r="G10" s="45"/>
+      <c r="H10" s="43"/>
+      <c r="I10" s="44"/>
+      <c r="J10" s="44"/>
+      <c r="K10" s="45"/>
       <c r="L10" s="4"/>
       <c r="M10" s="5"/>
       <c r="N10" s="5"/>
       <c r="O10" s="13"/>
       <c r="P10" s="6"/>
-      <c r="Q10" s="38" t="s">
+      <c r="Q10" s="24" t="s">
         <v>8</v>
       </c>
       <c r="R10" s="7" t="s">
@@ -1548,67 +1549,72 @@
       <c r="U10" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="V10" s="35" t="s">
+      <c r="V10" s="64" t="s">
         <v>13</v>
       </c>
-      <c r="W10" s="36"/>
+      <c r="W10" s="65"/>
     </row>
     <row r="11" spans="2:26" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="41" t="s">
+      <c r="B11" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="42"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="43"/>
-      <c r="F11" s="47" t="s">
+      <c r="C11" s="28"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="G11" s="48"/>
-      <c r="H11" s="48"/>
-      <c r="I11" s="48"/>
-      <c r="J11" s="48"/>
-      <c r="K11" s="49"/>
+      <c r="G11" s="34"/>
+      <c r="H11" s="34"/>
+      <c r="I11" s="34"/>
+      <c r="J11" s="34"/>
+      <c r="K11" s="35"/>
       <c r="L11" s="9"/>
       <c r="M11" s="9"/>
       <c r="N11" s="10"/>
       <c r="O11" s="14"/>
       <c r="P11" s="11"/>
-      <c r="Q11" s="39"/>
-      <c r="R11" s="50"/>
-      <c r="S11" s="52"/>
-      <c r="T11" s="50"/>
-      <c r="U11" s="50"/>
-      <c r="V11" s="62"/>
-      <c r="W11" s="63"/>
+      <c r="Q11" s="25"/>
+      <c r="R11" s="36"/>
+      <c r="S11" s="38"/>
+      <c r="T11" s="36"/>
+      <c r="U11" s="36"/>
+      <c r="V11" s="48"/>
+      <c r="W11" s="49"/>
     </row>
     <row r="12" spans="2:26" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="44"/>
-      <c r="C12" s="45"/>
-      <c r="D12" s="45"/>
-      <c r="E12" s="46"/>
-      <c r="F12" s="32" t="s">
+      <c r="B12" s="30"/>
+      <c r="C12" s="31"/>
+      <c r="D12" s="31"/>
+      <c r="E12" s="32"/>
+      <c r="F12" s="61" t="s">
         <v>16</v>
       </c>
-      <c r="G12" s="33"/>
-      <c r="H12" s="33"/>
-      <c r="I12" s="33"/>
-      <c r="J12" s="33"/>
-      <c r="K12" s="34"/>
+      <c r="G12" s="62"/>
+      <c r="H12" s="62"/>
+      <c r="I12" s="62"/>
+      <c r="J12" s="62"/>
+      <c r="K12" s="63"/>
       <c r="L12" s="9"/>
       <c r="M12" s="12"/>
       <c r="N12" s="9"/>
       <c r="O12" s="15"/>
       <c r="P12" s="11"/>
-      <c r="Q12" s="40"/>
-      <c r="R12" s="51"/>
-      <c r="S12" s="53"/>
-      <c r="T12" s="51"/>
-      <c r="U12" s="51"/>
-      <c r="V12" s="53"/>
-      <c r="W12" s="64"/>
+      <c r="Q12" s="26"/>
+      <c r="R12" s="37"/>
+      <c r="S12" s="39"/>
+      <c r="T12" s="37"/>
+      <c r="U12" s="37"/>
+      <c r="V12" s="39"/>
+      <c r="W12" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="L7:P7"/>
+    <mergeCell ref="Q7:W8"/>
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="F12:K12"/>
+    <mergeCell ref="V10:W10"/>
     <mergeCell ref="B2:Z2"/>
     <mergeCell ref="Q10:Q12"/>
     <mergeCell ref="B11:E12"/>
@@ -1625,11 +1631,6 @@
     <mergeCell ref="V11:W12"/>
     <mergeCell ref="C7:G7"/>
     <mergeCell ref="H7:K8"/>
-    <mergeCell ref="L7:P7"/>
-    <mergeCell ref="Q7:W8"/>
-    <mergeCell ref="C8:G8"/>
-    <mergeCell ref="F12:K12"/>
-    <mergeCell ref="V10:W10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>